<commit_message>
Actualización automática de clientes desde HubSpot
</commit_message>
<xml_diff>
--- a/clientes_hubspot.xlsx
+++ b/clientes_hubspot.xlsx
@@ -425,118 +425,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre Fiscal</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Contacto Principal</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Responsable Facturación</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Email Facturación</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Gestor Proyecto</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Email Proyecto</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Dominio/Web</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CIF</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Ciudad</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>createdate</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Email Facturación</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>email_responsable_de_gestion_del_proyecto</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>hs_lastmodifieddate</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>hs_object_id</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Empresa</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Contacto Principal</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>nombre_de_dominio_de_la_empresa</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Nombre Fiscal</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>nombre_responsable_degestion_del_proyecto</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Resp. Facturación</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mercadona</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Albertos.S.L</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>784597-G</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-30T14:32:27.639Z</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Alberto Perez</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Alberto</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>alberto@mercadona.es</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-30T15:09:01.116Z</t>
+          <t>Alberto</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>423832766666</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Mercadona</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+          <t>alberto@mercadona.es</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Benito Perez 85</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Elche</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>03201</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>